<commit_message>
Ajout dlv KIBO2/Épicerie – KB CHABRIOR MIELAK ETUI 375G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="14">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250390725817</t>
+  </si>
+  <si>
+    <t>60069630</t>
+  </si>
+  <si>
+    <t>KB CHABRIOR MIELAK ETUI 375G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>4008713711592</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>BOULES DE MAIS AU MIEL 375G BLONDOR</t>
-  </si>
-  <si>
-    <t/>
   </si>
 </sst>
 </file>
@@ -437,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -493,9 +502,32 @@
         <v>10</v>
       </c>
     </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -536,7 +568,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -577,6 +609,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – COTTERLEY INF.DU SOIR BIO 30G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="17">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250391947683</t>
+  </si>
+  <si>
+    <t>60070269</t>
+  </si>
+  <si>
+    <t>COTTERLEY INF.DU SOIR BIO 30G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250390725817</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>KB CHABRIOR MIELAK ETUI 375G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>4008713711592</t>
@@ -446,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -522,6 +531,29 @@
         <v>1</v>
       </c>
       <c r="G3" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – VINAIGRE BALSAMIQUE 500ML MILA FOOD
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="20">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3165351111922</t>
+  </si>
+  <si>
+    <t>50043029</t>
+  </si>
+  <si>
+    <t>VINAIGRE BALSAMIQUE 500ML MILA FOOD</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250391947683</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>COTTERLEY INF.DU SOIR BIO 30G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250390725817</t>
@@ -455,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -554,6 +563,29 @@
         <v>1</v>
       </c>
       <c r="G4" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – COTTERLEY THE VRT AGRUME25S40G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="23">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250392425838</t>
+  </si>
+  <si>
+    <t>60070283</t>
+  </si>
+  <si>
+    <t>COTTERLEY THE VRT AGRUME25S40G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3165351111922</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>VINAIGRE BALSAMIQUE 500ML MILA FOOD</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250391947683</t>
@@ -464,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -586,6 +595,29 @@
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – KB COTTERLEY CAMOMILLE 25S 22,5G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="26">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250390004356</t>
+  </si>
+  <si>
+    <t>60070318</t>
+  </si>
+  <si>
+    <t>KB COTTERLEY CAMOMILLE 25S 22,5G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250392425838</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>COTTERLEY THE VRT AGRUME25S40G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3165351111922</t>
@@ -473,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -618,6 +627,29 @@
         <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2">
+        <v>1</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – TOP BUDGET HUILE D OLIVE 1L
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="29">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250393444449</t>
+  </si>
+  <si>
+    <t>71083742</t>
+  </si>
+  <si>
+    <t>TOP BUDGET HUILE D OLIVE 1L</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250390004356</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>KB COTTERLEY CAMOMILLE 25S 22,5G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250392425838</t>
@@ -482,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -650,6 +659,29 @@
         <v>1</v>
       </c>
       <c r="G7" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – HUILE D'OLIVE 500ML BERTINI
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="32">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>6297000805306</t>
+  </si>
+  <si>
+    <t>71084515</t>
+  </si>
+  <si>
+    <t>HUILE D'OLIVE 500ML BERTINI</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250393444449</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>TOP BUDGET HUILE D OLIVE 1L</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250390004356</t>
@@ -491,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -682,6 +691,29 @@
         <v>1</v>
       </c>
       <c r="G8" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="2">
+        <v>1</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – T.BUDGET VINAIGRE ALCO.COL6D1L
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="35">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3410280010458</t>
+  </si>
+  <si>
+    <t>60068683</t>
+  </si>
+  <si>
+    <t>T.BUDGET VINAIGRE ALCO.COL6D1L</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>6297000805306</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>HUILE D'OLIVE 500ML BERTINI</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250393444449</t>
@@ -500,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -714,6 +723,29 @@
         <v>1</v>
       </c>
       <c r="G9" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="2">
+        <v>1</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – TB.VINAIGRE ALCO.CRIST 8 1,5L
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="38">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3410280142227</t>
+  </si>
+  <si>
+    <t>71081943</t>
+  </si>
+  <si>
+    <t>TB.VINAIGRE ALCO.CRIST 8 1,5L</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3410280010458</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>T.BUDGET VINAIGRE ALCO.COL6D1L</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>6297000805306</t>
@@ -509,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -746,6 +755,29 @@
         <v>1</v>
       </c>
       <c r="G10" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="2">
+        <v>1</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – LESIEUR MAYONNAISE 235G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="41">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3265478891001</t>
+  </si>
+  <si>
+    <t>50067605</t>
+  </si>
+  <si>
+    <t>LESIEUR MAYONNAISE 235G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3410280142227</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>TB.VINAIGRE ALCO.CRIST 8 1,5L</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3410280010458</t>
@@ -518,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -778,6 +787,29 @@
         <v>1</v>
       </c>
       <c r="G11" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="2">
+        <v>1</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – LESIEUR MAYONNAISE 475G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="44">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3265478892008</t>
+  </si>
+  <si>
+    <t>50067606</t>
+  </si>
+  <si>
+    <t>LESIEUR MAYONNAISE 475G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3265478891001</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>LESIEUR MAYONNAISE 235G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3410280142227</t>
@@ -527,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -810,6 +819,29 @@
         <v>1</v>
       </c>
       <c r="G12" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="2">
+        <v>1</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – KB BOUTON OR KETCHUP NAT SPL.560G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="47">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250390115656</t>
+  </si>
+  <si>
+    <t>60069930</t>
+  </si>
+  <si>
+    <t>KB BOUTON OR KETCHUP NAT SPL.560G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3265478892008</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>LESIEUR MAYONNAISE 475G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3265478891001</t>
@@ -536,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -842,6 +851,29 @@
         <v>1</v>
       </c>
       <c r="G13" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="2">
+        <v>1</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – TOP BUDGET PUREE DE TOMATE500G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="50">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3410280141886</t>
+  </si>
+  <si>
+    <t>60077136</t>
+  </si>
+  <si>
+    <t>TOP BUDGET PUREE DE TOMATE500G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250390115656</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>KB BOUTON OR KETCHUP NAT SPL.560G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3265478892008</t>
@@ -545,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -874,6 +883,29 @@
         <v>1</v>
       </c>
       <c r="G14" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="2">
+        <v>1</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – KB TOP BUDGET MX N°4 1KG
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="53">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3410280043678</t>
+  </si>
+  <si>
+    <t>60068377</t>
+  </si>
+  <si>
+    <t>KB TOP BUDGET MX N°4 1KG</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3410280141886</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>TOP BUDGET PUREE DE TOMATE500G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250390115656</t>
@@ -554,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -906,6 +915,29 @@
         <v>1</v>
       </c>
       <c r="G15" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="2">
+        <v>1</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – KB CHAB.SUCR.MORCEAUX BLC N4 1KG
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="56">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250392035068</t>
+  </si>
+  <si>
+    <t>60069049</t>
+  </si>
+  <si>
+    <t>KB CHAB.SUCR.MORCEAUX BLC N4 1KG</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3410280043678</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>KB TOP BUDGET MX N°4 1KG</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3410280141886</t>
@@ -563,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -938,6 +947,29 @@
         <v>1</v>
       </c>
       <c r="G16" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" s="2">
+        <v>1</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – CHABRIOR SPRITS BEURRE 400G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="59">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250391612635</t>
+  </si>
+  <si>
+    <t>60069099</t>
+  </si>
+  <si>
+    <t>CHABRIOR SPRITS BEURRE 400G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250392035068</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>KB CHAB.SUCR.MORCEAUX BLC N4 1KG</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3410280043678</t>
@@ -572,7 +581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -970,6 +979,29 @@
         <v>1</v>
       </c>
       <c r="G17" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="2">
+        <v>1</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – GOFRETY VANILLE 4
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="62">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>6161105492719</t>
+  </si>
+  <si>
+    <t>60071021</t>
+  </si>
+  <si>
+    <t>GOFRETY VANILLE 4</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250391612635</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>CHABRIOR SPRITS BEURRE 400G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250392035068</t>
@@ -581,7 +590,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1002,6 +1011,29 @@
         <v>1</v>
       </c>
       <c r="G18" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="2">
+        <v>1</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – IDS NOUILLE ASIAT.250GRS
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="65">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250390325178</t>
+  </si>
+  <si>
+    <t>60070234</t>
+  </si>
+  <si>
+    <t>IDS NOUILLE ASIAT.250GRS</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>6161105492719</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>GOFRETY VANILLE 4</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250391612635</t>
@@ -590,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1034,6 +1043,29 @@
         <v>1</v>
       </c>
       <c r="G19" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="2">
+        <v>1</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – HUILE DE PEPINS DE RAISINS 1 L
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="68">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3281712000015</t>
+  </si>
+  <si>
+    <t>71085057</t>
+  </si>
+  <si>
+    <t>HUILE DE PEPINS DE RAISINS 1 L</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250390325178</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>IDS NOUILLE ASIAT.250GRS</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>6161105492719</t>
@@ -599,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1066,6 +1075,29 @@
         <v>1</v>
       </c>
       <c r="G20" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="2">
+        <v>1</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – BO CREA HUILE NOISETTE 25CL
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="71">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250391650132</t>
+  </si>
+  <si>
+    <t>60069114</t>
+  </si>
+  <si>
+    <t>BO CREA HUILE NOISETTE 25CL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3281712000015</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>HUILE DE PEPINS DE RAISINS 1 L</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250390325178</t>
@@ -608,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1098,6 +1107,29 @@
         <v>1</v>
       </c>
       <c r="G21" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="2">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – LES CREATION HUIL SESAME 25CL
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="74">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250392850685</t>
+  </si>
+  <si>
+    <t>71085568</t>
+  </si>
+  <si>
+    <t>LES CREATION HUIL SESAME 25CL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250391650132</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>BO CREA HUILE NOISETTE 25CL</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3281712000015</t>
@@ -617,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1130,6 +1139,29 @@
         <v>1</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="2">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – LES CREATIONS HUILE NOIX 25CL
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="77">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250392257217</t>
+  </si>
+  <si>
+    <t>60068947</t>
+  </si>
+  <si>
+    <t>LES CREATIONS HUILE NOIX 25CL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250392850685</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>LES CREATION HUIL SESAME 25CL</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250391650132</t>
@@ -626,7 +635,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1162,6 +1171,29 @@
         <v>1</v>
       </c>
       <c r="G23" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="2">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – BO MOUTARDE DIJON SQUEZER 265G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="80">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250391413850</t>
+  </si>
+  <si>
+    <t>60069294</t>
+  </si>
+  <si>
+    <t>BO MOUTARDE DIJON SQUEZER 265G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250392257217</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>LES CREATIONS HUILE NOIX 25CL</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250392850685</t>
@@ -635,7 +644,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1194,6 +1203,29 @@
         <v>1</v>
       </c>
       <c r="G24" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" s="2">
+        <v>1</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – ST ELOI SOUPE MOUL 9LEG 75G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="83">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250390111665</t>
+  </si>
+  <si>
+    <t>60069910</t>
+  </si>
+  <si>
+    <t>ST ELOI SOUPE MOUL 9LEG 75G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250391413850</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>BO MOUTARDE DIJON SQUEZER 265G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250392257217</t>
@@ -644,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1226,6 +1235,29 @@
         <v>1</v>
       </c>
       <c r="G25" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" s="2">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – BOUT.OR SAUCE TARTARE PT 235G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="86">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250390109396</t>
+  </si>
+  <si>
+    <t>60069898</t>
+  </si>
+  <si>
+    <t>BOUT.OR SAUCE TARTARE PT 235G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250391413850</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>BO MOUTARDE DIJON SQUEZER 265G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250390111665</t>
@@ -653,7 +662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -734,13 +743,13 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>10</v>
@@ -757,13 +766,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>10</v>
@@ -1281,6 +1290,29 @@
         <v>1</v>
       </c>
       <c r="G27" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F28" s="2">
+        <v>1</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – BOUT.OR SCE BEARNAISE PT 235G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="89">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250390109389</t>
+  </si>
+  <si>
+    <t>60069897</t>
+  </si>
+  <si>
+    <t>BOUT.OR SCE BEARNAISE PT 235G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250390109396</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>BOUT.OR SAUCE TARTARE PT 235G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250391413850</t>
@@ -662,7 +671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -766,13 +775,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>10</v>
@@ -789,13 +798,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>
@@ -1313,6 +1322,29 @@
         <v>1</v>
       </c>
       <c r="G28" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" s="2">
+        <v>1</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – BOUTON D OR HUILE PIZZA 250ML
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="92">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250390139393</t>
+  </si>
+  <si>
+    <t>60069768</t>
+  </si>
+  <si>
+    <t>BOUTON D OR HUILE PIZZA 250ML</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250390109389</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>BOUT.OR SCE BEARNAISE PT 235G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250390109396</t>
@@ -671,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -798,13 +807,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>
@@ -821,13 +830,13 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>10</v>
@@ -1345,6 +1354,29 @@
         <v>1</v>
       </c>
       <c r="G29" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" s="2">
+        <v>1</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – IVORIA PATE A TARTINER 200G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="96">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,21 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250392397029</t>
+  </si>
+  <si>
+    <t>71085598</t>
+  </si>
+  <si>
+    <t>IVORIA PATE A TARTINER 200G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-11-30</t>
+  </si>
+  <si>
     <t>3250390139393</t>
   </si>
   <si>
@@ -43,9 +58,6 @@
   </si>
   <si>
     <t>BOUTON D OR HUILE PIZZA 250ML</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>3250390109389</t>
@@ -680,7 +692,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -723,28 +735,28 @@
       <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>10</v>
+      <c r="D2" s="2">
+        <v>14500</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F2" s="2">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>10</v>
@@ -761,13 +773,13 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>10</v>
@@ -784,13 +796,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>10</v>
@@ -807,13 +819,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>
@@ -830,13 +842,13 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>10</v>
@@ -853,13 +865,13 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>10</v>
@@ -876,13 +888,13 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>10</v>
@@ -899,13 +911,13 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
@@ -922,13 +934,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>10</v>
@@ -945,13 +957,13 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>10</v>
@@ -968,13 +980,13 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>10</v>
@@ -991,13 +1003,13 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>10</v>
@@ -1014,13 +1026,13 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>10</v>
@@ -1037,13 +1049,13 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
@@ -1060,13 +1072,13 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>10</v>
@@ -1083,13 +1095,13 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>10</v>
@@ -1106,13 +1118,13 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>10</v>
@@ -1129,13 +1141,13 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>10</v>
@@ -1152,13 +1164,13 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>10</v>
@@ -1175,13 +1187,13 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>10</v>
@@ -1198,13 +1210,13 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>10</v>
@@ -1221,13 +1233,13 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>10</v>
@@ -1244,13 +1256,13 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>10</v>
@@ -1267,13 +1279,13 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>10</v>
@@ -1290,13 +1302,13 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>10</v>
@@ -1313,13 +1325,13 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>10</v>
@@ -1336,13 +1348,13 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>10</v>
@@ -1359,13 +1371,13 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>10</v>
@@ -1377,6 +1389,29 @@
         <v>1</v>
       </c>
       <c r="G30" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" s="2">
+        <v>1</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – ⚠️ HORS BASE
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="97">
   <si>
     <t>Code Barre</t>
   </si>
@@ -39,13 +39,16 @@
     <t>3250392397029</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>⚠️ HORS BASE</t>
+  </si>
+  <si>
     <t>71085598</t>
   </si>
   <si>
     <t>IVORIA PATE A TARTINER 200G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>2026-11-30</t>
@@ -692,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -735,684 +738,707 @@
       <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2">
-        <v>14500</v>
+      <c r="D2" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F2" s="2">
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="2">
+        <v>14500</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2">
+        <v>71</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F4" s="2">
         <v>1</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F5" s="2">
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F6" s="2">
         <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F7" s="2">
         <v>1</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F8" s="2">
         <v>1</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F9" s="2">
         <v>1</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F10" s="2">
         <v>1</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F11" s="2">
         <v>1</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="D12" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F12" s="2">
         <v>1</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="D13" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F13" s="2">
         <v>1</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="D14" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F14" s="2">
         <v>1</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="D15" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F15" s="2">
         <v>1</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="D16" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F16" s="2">
         <v>1</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="D17" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F17" s="2">
         <v>1</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="D18" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F18" s="2">
         <v>1</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="D19" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F19" s="2">
         <v>1</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>62</v>
-      </c>
       <c r="D20" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F20" s="2">
         <v>1</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="D21" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F21" s="2">
         <v>1</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="D22" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F22" s="2">
         <v>1</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="D23" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F23" s="2">
         <v>1</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="D24" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F24" s="2">
         <v>1</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="D25" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F25" s="2">
         <v>1</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="D26" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F26" s="2">
         <v>1</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>83</v>
-      </c>
       <c r="D27" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F27" s="2">
         <v>1</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="D28" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F28" s="2">
         <v>1</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="D29" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F29" s="2">
         <v>1</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="D30" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F30" s="2">
         <v>1</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="D31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F31" s="2">
+        <v>1</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F31" s="2">
-        <v>1</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>10</v>
+      <c r="C32" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F32" s="2">
+        <v>1</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – IVORIA PATE TARTINER DUO 400G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="100">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,21 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3250391062126</t>
+  </si>
+  <si>
+    <t>60069551</t>
+  </si>
+  <si>
+    <t>IVORIA PATE TARTINER DUO 400G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-11-30</t>
+  </si>
+  <si>
     <t>3250392397029</t>
   </si>
   <si>
@@ -43,12 +58,6 @@
   </si>
   <si>
     <t>IVORIA PATE A TARTINER 200G</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>2026-11-30</t>
   </si>
   <si>
     <t>⚠️ HORS BASE</t>
@@ -695,7 +704,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -738,14 +747,14 @@
       <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>10</v>
+      <c r="D2" s="2">
+        <v>19900</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F2" s="2">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>11</v>
@@ -753,13 +762,13 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>10</v>
@@ -768,56 +777,56 @@
         <v>10</v>
       </c>
       <c r="F3" s="2">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="2">
-        <v>14500</v>
+        <v>15</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F4" s="2">
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>10</v>
+      <c r="D5" s="2">
+        <v>14500</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F5" s="2">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -914,13 +923,13 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
@@ -937,13 +946,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>10</v>
@@ -1461,6 +1470,29 @@
         <v>1</v>
       </c>
       <c r="G33" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" s="2">
+        <v>1</v>
+      </c>
+      <c r="G34" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout dlv KIBO2/Épicerie – LAIT EN POUDRE O LAIT 250 G
</commit_message>
<xml_diff>
--- a/dlv_KIBO2.xlsx
+++ b/dlv_KIBO2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="103">
   <si>
     <t>Code Barre</t>
   </si>
@@ -36,6 +36,18 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3700005095038</t>
+  </si>
+  <si>
+    <t>50044462</t>
+  </si>
+  <si>
+    <t>LAIT EN POUDRE O LAIT 250 G</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>3250391062126</t>
   </si>
   <si>
@@ -43,9 +55,6 @@
   </si>
   <si>
     <t>IVORIA PATE TARTINER DUO 400G</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>2026-11-30</t>
@@ -704,7 +713,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -747,51 +756,51 @@
       <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2">
-        <v>19900</v>
+      <c r="D2" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F2" s="2">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2">
+        <v>19900</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="2">
+        <v>16</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="2">
-        <v>71</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>10</v>
@@ -800,56 +809,56 @@
         <v>10</v>
       </c>
       <c r="F4" s="2">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="2">
-        <v>14500</v>
+        <v>18</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F5" s="2">
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>10</v>
+      <c r="D6" s="2">
+        <v>14500</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F6" s="2">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -946,13 +955,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>10</v>
@@ -969,13 +978,13 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>10</v>
@@ -1493,6 +1502,29 @@
         <v>1</v>
       </c>
       <c r="G34" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" s="2">
+        <v>1</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>